<commit_message>
atualização de mapa de localização
</commit_message>
<xml_diff>
--- a/R Markdown/resultados/df_integrado_2025.xlsx
+++ b/R Markdown/resultados/df_integrado_2025.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:M33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -372,45 +372,50 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>populacao</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>valor</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ano</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>idrgp_real</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>idrgp_diferenca</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>idrgp_var_percentual</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>valor_previsto</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>status_valor</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>status_var_percentual</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>status_estatistico</t>
         </is>
@@ -431,34 +436,37 @@
         <v>0.05427611013661751</v>
       </c>
       <c r="D2">
+        <v>412804</v>
+      </c>
+      <c r="E2">
         <v>1688434491</v>
       </c>
-      <c r="E2">
-        <v>2025</v>
-      </c>
       <c r="F2">
+        <v>2025</v>
+      </c>
+      <c r="G2">
         <v>0.02953342009533873</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>-0.02474269004127878</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>-0.455867046827773</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>3102981506.921495</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -479,34 +487,37 @@
         <v>0.0768001000600067</v>
       </c>
       <c r="D3">
+        <v>570809</v>
+      </c>
+      <c r="E3">
         <v>3036975936.59</v>
       </c>
-      <c r="E3">
-        <v>2025</v>
-      </c>
       <c r="F3">
+        <v>2025</v>
+      </c>
+      <c r="G3">
         <v>0.05312156712791723</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>-0.02367853293208947</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>-0.3083138291953861</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>4390684771.183432</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -527,34 +538,37 @@
         <v>0.01518693116727706</v>
       </c>
       <c r="D4">
+        <v>354316</v>
+      </c>
+      <c r="E4">
         <v>2415839399.78</v>
       </c>
-      <c r="E4">
-        <v>2025</v>
-      </c>
       <c r="F4">
+        <v>2025</v>
+      </c>
+      <c r="G4">
         <v>0.0422568955188287</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>0.02706996435155164</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>1.78245124399317</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>868241413.0329791</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -575,34 +589,37 @@
         <v>0.02852737800077722</v>
       </c>
       <c r="D5">
+        <v>480878</v>
+      </c>
+      <c r="E5">
         <v>1586731737.63</v>
       </c>
-      <c r="E5">
-        <v>2025</v>
-      </c>
       <c r="F5">
+        <v>2025</v>
+      </c>
+      <c r="G5">
         <v>0.02775447625349036</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>-0.0007729017472868603</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>-0.02709333284207903</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>1630918762.500827</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -623,34 +640,37 @@
         <v>0.01196759457375883</v>
       </c>
       <c r="D6">
+        <v>338347</v>
+      </c>
+      <c r="E6">
         <v>1635541987.13</v>
       </c>
-      <c r="E6">
-        <v>2025</v>
-      </c>
       <c r="F6">
+        <v>2025</v>
+      </c>
+      <c r="G6">
         <v>0.02860824559492808</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>0.01664065102116925</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1.390475831931753</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>684190973.7310801</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -671,34 +691,37 @@
         <v>0.0146420577822676</v>
       </c>
       <c r="D7">
+        <v>214958</v>
+      </c>
+      <c r="E7">
         <v>1532982112.9</v>
       </c>
-      <c r="E7">
-        <v>2025</v>
-      </c>
       <c r="F7">
+        <v>2025</v>
+      </c>
+      <c r="G7">
         <v>0.0268143093381736</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>0.012172251555906</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>0.8313210982302859</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>837090838.0738972</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -719,34 +742,37 @@
         <v>0.03106350078710079</v>
       </c>
       <c r="D8">
+        <v>276378</v>
+      </c>
+      <c r="E8">
         <v>1001849833.82</v>
       </c>
-      <c r="E8">
-        <v>2025</v>
-      </c>
       <c r="F8">
+        <v>2025</v>
+      </c>
+      <c r="G8">
         <v>0.01752395616908264</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>-0.01353954461801815</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>-0.4358666690793745</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>1775909663.385874</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -767,34 +793,37 @@
         <v>0.00780842708567104</v>
       </c>
       <c r="D9">
+        <v>272332</v>
+      </c>
+      <c r="E9">
         <v>1665436605.22</v>
       </c>
-      <c r="E9">
-        <v>2025</v>
-      </c>
       <c r="F9">
+        <v>2025</v>
+      </c>
+      <c r="G9">
         <v>0.02913115028524791</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>0.02132272319957687</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>2.730732190444017</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>446410120.1061517</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -815,34 +844,37 @@
         <v>0.02854078087441063</v>
       </c>
       <c r="D10">
+        <v>266715</v>
+      </c>
+      <c r="E10">
         <v>1078636355.45</v>
       </c>
-      <c r="E10">
-        <v>2025</v>
-      </c>
       <c r="F10">
+        <v>2025</v>
+      </c>
+      <c r="G10">
         <v>0.01886707526138185</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>-0.009673705613028775</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>-0.3389432705291578</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>1631685008.809182</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -863,34 +895,37 @@
         <v>0.03997675152969091</v>
       </c>
       <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
         <v>1362970185.21</v>
       </c>
-      <c r="E11">
-        <v>2025</v>
-      </c>
       <c r="F11">
+        <v>2025</v>
+      </c>
+      <c r="G11">
         <v>0.02384052876898294</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>-0.01613622276070797</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>-0.4036401694300631</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>2285482883.559443</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -911,34 +946,37 @@
         <v>0.03619588619759224</v>
       </c>
       <c r="D12">
+        <v>283892</v>
+      </c>
+      <c r="E12">
         <v>1078973096.78</v>
       </c>
-      <c r="E12">
-        <v>2025</v>
-      </c>
       <c r="F12">
+        <v>2025</v>
+      </c>
+      <c r="G12">
         <v>0.01887296540590055</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>-0.01732292079169168</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>-0.478588110735192</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>2069329677.735877</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -959,34 +997,37 @@
         <v>0.02290605900133662</v>
       </c>
       <c r="D13">
+        <v>306275</v>
+      </c>
+      <c r="E13">
         <v>990146048.22</v>
       </c>
-      <c r="E13">
-        <v>2025</v>
-      </c>
       <c r="F13">
+        <v>2025</v>
+      </c>
+      <c r="G13">
         <v>0.01731923823736954</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>-0.005586820763967076</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>-0.2439014395117499</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>1309546268.122259</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1007,34 +1048,37 @@
         <v>0.07049848664210395</v>
       </c>
       <c r="D14">
+        <v>675598</v>
+      </c>
+      <c r="E14">
         <v>2562583888.81</v>
       </c>
-      <c r="E14">
-        <v>2025</v>
-      </c>
       <c r="F14">
+        <v>2025</v>
+      </c>
+      <c r="G14">
         <v>0.04482369136687609</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>-0.02567479527522786</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>-0.3641893109786849</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>4030419640.718074</v>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -1055,34 +1099,37 @@
         <v>0.03440060917127755</v>
       </c>
       <c r="D15">
+        <v>372134</v>
+      </c>
+      <c r="E15">
         <v>1202924802.61</v>
       </c>
-      <c r="E15">
-        <v>2025</v>
-      </c>
       <c r="F15">
+        <v>2025</v>
+      </c>
+      <c r="G15">
         <v>0.02104107901606681</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>-0.01335953015521073</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>-0.3883515576336115</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>1966693151.307702</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -1103,34 +1150,37 @@
         <v>0.03138103348631988</v>
       </c>
       <c r="D16">
+        <v>468522</v>
+      </c>
+      <c r="E16">
         <v>2120033849.32</v>
       </c>
-      <c r="E16">
-        <v>2025</v>
-      </c>
       <c r="F16">
+        <v>2025</v>
+      </c>
+      <c r="G16">
         <v>0.03708278326583037</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>0.00570174977951049</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>0.181694136427855</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>1794063103.104373</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1151,34 +1201,37 @@
         <v>0.01774539803593836</v>
       </c>
       <c r="D17">
+        <v>423536</v>
+      </c>
+      <c r="E17">
         <v>6837566518.55</v>
       </c>
-      <c r="E17">
-        <v>2025</v>
-      </c>
       <c r="F17">
+        <v>2025</v>
+      </c>
+      <c r="G17">
         <v>0.1195999758939773</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>0.101854577858039</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>5.739774202402272</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>1014509731.81162</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -1199,34 +1252,37 @@
         <v>0.04982071041328871</v>
       </c>
       <c r="D18">
+        <v>501306</v>
+      </c>
+      <c r="E18">
         <v>2039768606.41</v>
       </c>
-      <c r="E18">
-        <v>2025</v>
-      </c>
       <c r="F18">
+        <v>2025</v>
+      </c>
+      <c r="G18">
         <v>0.03567881577372384</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>-0.01414189463956487</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>-0.2838557403587885</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>2848264967.496807</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -1247,34 +1303,37 @@
         <v>0.05776210461891745</v>
       </c>
       <c r="D19">
+        <v>453527</v>
+      </c>
+      <c r="E19">
         <v>1956937590.38</v>
       </c>
-      <c r="E19">
-        <v>2025</v>
-      </c>
       <c r="F19">
+        <v>2025</v>
+      </c>
+      <c r="G19">
         <v>0.03422996880549536</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>-0.02353213581342209</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>-0.4073974791721001</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>3302276857.759642</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -1295,34 +1354,37 @@
         <v>0.021319194803451</v>
       </c>
       <c r="D20">
+        <v>163083</v>
+      </c>
+      <c r="E20">
         <v>918890507.58</v>
       </c>
-      <c r="E20">
-        <v>2025</v>
-      </c>
       <c r="F20">
+        <v>2025</v>
+      </c>
+      <c r="G20">
         <v>0.01607286485003414</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>-0.00524632995341686</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>-0.246084807694877</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>1218824765.64832</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1343,34 +1405,37 @@
         <v>0.02476472440077774</v>
       </c>
       <c r="D21">
+        <v>187216</v>
+      </c>
+      <c r="E21">
         <v>1335237845.73</v>
       </c>
-      <c r="E21">
-        <v>2025</v>
-      </c>
       <c r="F21">
+        <v>2025</v>
+      </c>
+      <c r="G21">
         <v>0.02335544579036864</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>-0.001409278610409095</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>-0.05690669468402548</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>1415806726.867435</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1391,34 +1456,37 @@
         <v>0.007949529934269608</v>
       </c>
       <c r="D22">
+        <v>337654</v>
+      </c>
+      <c r="E22">
         <v>1939351672.66</v>
       </c>
-      <c r="E22">
-        <v>2025</v>
-      </c>
       <c r="F22">
+        <v>2025</v>
+      </c>
+      <c r="G22">
         <v>0.0339223629738476</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>0.02597283303957799</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>3.267216207037825</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>454477012.3110872</v>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -1439,34 +1507,37 @@
         <v>0.01470567515443555</v>
       </c>
       <c r="D23">
+        <v>243728</v>
+      </c>
+      <c r="E23">
         <v>776448481.35</v>
       </c>
-      <c r="E23">
-        <v>2025</v>
-      </c>
       <c r="F23">
+        <v>2025</v>
+      </c>
+      <c r="G23">
         <v>0.01358132595864943</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>-0.001124349195786129</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>-0.07645682255173442</v>
       </c>
-      <c r="I23">
+      <c r="J23">
         <v>840727862.3348334</v>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1487,34 +1558,37 @@
         <v>0.006306371387863901</v>
       </c>
       <c r="D24">
+        <v>285815</v>
+      </c>
+      <c r="E24">
         <v>997429393.05</v>
       </c>
-      <c r="E24">
-        <v>2025</v>
-      </c>
       <c r="F24">
+        <v>2025</v>
+      </c>
+      <c r="G24">
         <v>0.01744663558900514</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>0.01114026420114124</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>1.766509378527845</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>360537145.0360911</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -1535,34 +1609,37 @@
         <v>0.04188065349285796</v>
       </c>
       <c r="D25">
+        <v>165138</v>
+      </c>
+      <c r="E25">
         <v>1294481417.88</v>
       </c>
-      <c r="E25">
-        <v>2025</v>
-      </c>
       <c r="F25">
+        <v>2025</v>
+      </c>
+      <c r="G25">
         <v>0.0226425506726158</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>-0.01923810282024216</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>-0.4593553637725089</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>2394329530.230114</v>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>
@@ -1583,34 +1660,37 @@
         <v>0.03550998362496413</v>
       </c>
       <c r="D26">
+        <v>480218</v>
+      </c>
+      <c r="E26">
         <v>1785675753.86</v>
       </c>
-      <c r="E26">
-        <v>2025</v>
-      </c>
       <c r="F26">
+        <v>2025</v>
+      </c>
+      <c r="G26">
         <v>0.03123432533149316</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>-0.004275658293470971</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>-0.1204072167035614</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>2030116421.792191</v>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1631,34 +1711,37 @@
         <v>0.04493881006046815</v>
       </c>
       <c r="D27">
+        <v>380513</v>
+      </c>
+      <c r="E27">
         <v>2301085241.03</v>
       </c>
-      <c r="E27">
-        <v>2025</v>
-      </c>
       <c r="F27">
+        <v>2025</v>
+      </c>
+      <c r="G27">
         <v>0.04024966171964013</v>
       </c>
-      <c r="G27">
+      <c r="H27">
         <v>-0.004689148340828016</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>-0.1043451825831271</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>2569165259.074339</v>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1679,34 +1762,37 @@
         <v>0.03328667005479251</v>
       </c>
       <c r="D28">
+        <v>469766</v>
+      </c>
+      <c r="E28">
         <v>1705356170.99</v>
       </c>
-      <c r="E28">
-        <v>2025</v>
-      </c>
       <c r="F28">
+        <v>2025</v>
+      </c>
+      <c r="G28">
         <v>0.02982940734656313</v>
       </c>
-      <c r="G28">
+      <c r="H28">
         <v>-0.003457262708229381</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>-0.1038632792808187</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>1903008917.680989</v>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1727,34 +1813,37 @@
         <v>0.01278087722546964</v>
       </c>
       <c r="D29">
+        <v>266497</v>
+      </c>
+      <c r="E29">
         <v>989484961.0599999</v>
       </c>
-      <c r="E29">
-        <v>2025</v>
-      </c>
       <c r="F29">
+        <v>2025</v>
+      </c>
+      <c r="G29">
         <v>0.01730767476545518</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>0.004526797539985538</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>0.3541851987252149</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>730686587.0277332</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1775,34 +1864,37 @@
         <v>0.01442360309469943</v>
       </c>
       <c r="D30">
+        <v>318913</v>
+      </c>
+      <c r="E30">
         <v>1376552981.17</v>
       </c>
-      <c r="E30">
-        <v>2025</v>
-      </c>
       <c r="F30">
+        <v>2025</v>
+      </c>
+      <c r="G30">
         <v>0.0240781135975885</v>
       </c>
-      <c r="G30">
+      <c r="H30">
         <v>0.009654510502889065</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>0.6693549759724757</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>824601718.0187185</v>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -1823,34 +1915,37 @@
         <v>0.01471389456597418</v>
       </c>
       <c r="D31">
+        <v>276069</v>
+      </c>
+      <c r="E31">
         <v>1594437761.49</v>
       </c>
-      <c r="E31">
-        <v>2025</v>
-      </c>
       <c r="F31">
+        <v>2025</v>
+      </c>
+      <c r="G31">
         <v>0.02788926693748503</v>
       </c>
-      <c r="G31">
+      <c r="H31">
         <v>0.01317537237151085</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>0.8954374596362024</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>841197768.5594679</v>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Acima do IDRGP Alvo</t>
         </is>
@@ -1871,34 +1966,37 @@
         <v>0.01564514619986043</v>
       </c>
       <c r="D32">
+        <v>203874</v>
+      </c>
+      <c r="E32">
         <v>1144062973.34</v>
       </c>
-      <c r="E32">
-        <v>2025</v>
-      </c>
       <c r="F32">
+        <v>2025</v>
+      </c>
+      <c r="G32">
         <v>0.02001149146577848</v>
       </c>
-      <c r="G32">
+      <c r="H32">
         <v>0.004366345265918049</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>0.2790862552602417</v>
       </c>
-      <c r="I32">
+      <c r="J32">
         <v>894437703.9742563</v>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Valor previsto (R$) superado</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Dentro do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>Dentro do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
         <is>
           <t>Dentro do IDRGP Alvo</t>
         </is>
@@ -1919,34 +2017,37 @@
         <v>0.08227494643576272</v>
       </c>
       <c r="D33">
+        <v>605383</v>
+      </c>
+      <c r="E33">
         <v>3217471932.62</v>
       </c>
-      <c r="E33">
-        <v>2025</v>
-      </c>
       <c r="F33">
+        <v>2025</v>
+      </c>
+      <c r="G33">
         <v>0.05627873082286368</v>
       </c>
-      <c r="G33">
+      <c r="H33">
         <v>-0.02599621561289904</v>
       </c>
-      <c r="H33">
+      <c r="I33">
         <v>-0.3159675786990143</v>
       </c>
-      <c r="I33">
+      <c r="J33">
         <v>4703683381.703713</v>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Valor previsto (R$) não atingido</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Abaixo do IDRGP Alvo</t>
-        </is>
-      </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>Abaixo do IDRGP Alvo</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
         <is>
           <t>Abaixo do IDRGP Alvo</t>
         </is>

</xml_diff>